<commit_message>
fix: persist gateway health and staged write rows
</commit_message>
<xml_diff>
--- a/outputs/issue-2/KKB_V2_CONFIG_BASELINE.xlsx
+++ b/outputs/issue-2/KKB_V2_CONFIG_BASELINE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SCHEMA" sheetId="1" r:id="Re51ce325b0d74aab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_VERSION" sheetId="2" r:id="R68f2536b91734ea7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_GLOBAL" sheetId="3" r:id="R127a4754ebd54b50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_BRANCH" sheetId="4" r:id="R6e27ae6bccac4323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_USER" sheetId="5" r:id="R746b8643de30404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_THONG_BAO" sheetId="6" r:id="R5d198937e77f4174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SNAPSHOT" sheetId="7" r:id="R9c97cfbab33b40e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERATION" sheetId="8" r:id="R1cdd3fae763e4565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERROR_BIA" sheetId="9" r:id="Re6517aa200e645e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SCHEMA" sheetId="1" r:id="Rff5ee20d738c4112"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_VERSION" sheetId="2" r:id="R3ed994e67de340b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_GLOBAL" sheetId="3" r:id="R0c681aac3625444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_BRANCH" sheetId="4" r:id="Rdd6e309094254020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_USER" sheetId="5" r:id="R49de009770c54ac8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_THONG_BAO" sheetId="6" r:id="R4e3ee4fb76f6474f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SNAPSHOT" sheetId="7" r:id="R7a5890ca5b0a4f91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERATION" sheetId="8" r:id="R6757e33456b64429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERROR_BIA" sheetId="9" r:id="R210f965374cb4883"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3073,10 +3073,10 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="9" t="str">
-        <x:v>STATUS_CONFIG_LINE</x:v>
+        <x:v>STATUS_GATEWAY_HEALTH_LINE</x:v>
       </x:c>
       <x:c r="B3" s="9" t="str">
-        <x:v>Cấu hình: {config_version}</x:v>
+        <x:v>Config Gateway: {gateway_health}</x:v>
       </x:c>
       <x:c r="C3" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3087,10 +3087,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
-        <x:v>STATUS_BRANCH_COUNT_LINE</x:v>
+        <x:v>STATUS_CONFIG_LINE</x:v>
       </x:c>
       <x:c r="B4" s="9" t="str">
-        <x:v>Chi nhánh hoạt động: {active_branch_count}</x:v>
+        <x:v>Cấu hình: {config_version}</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3101,10 +3101,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="9" t="str">
-        <x:v>STATUS_BRANCH_LINE</x:v>
+        <x:v>STATUS_BRANCH_COUNT_LINE</x:v>
       </x:c>
       <x:c r="B5" s="9" t="str">
-        <x:v>- {branch_name} ({branch_id})</x:v>
+        <x:v>Chi nhánh hoạt động: {active_branch_count}</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3115,10 +3115,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="9" t="str">
-        <x:v>STATUS_MAINTENANCE_LINE</x:v>
+        <x:v>STATUS_BRANCH_LINE</x:v>
       </x:c>
       <x:c r="B6" s="9" t="str">
-        <x:v>Bảo trì cấu hình: {maintenance_mode}</x:v>
+        <x:v>- {branch_name} ({branch_id})</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3129,10 +3129,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="9" t="str">
-        <x:v>ERROR_GENERIC</x:v>
+        <x:v>STATUS_MAINTENANCE_LINE</x:v>
       </x:c>
       <x:c r="B7" s="9" t="str">
-        <x:v>Không thể hoàn tất thao tác. Mã lỗi: {error_id}</x:v>
+        <x:v>Bảo trì cấu hình: {maintenance_mode}</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3143,10 +3143,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
-        <x:v>USER_NOT_ACTIVE</x:v>
+        <x:v>ERROR_GENERIC</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>Tài khoản chưa được cấp quyền hoạt động. Mã lỗi: {error_id}</x:v>
+        <x:v>Không thể hoàn tất thao tác. Mã lỗi: {error_id}</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3157,10 +3157,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="9" t="str">
-        <x:v>COMMAND_NOT_AVAILABLE</x:v>
+        <x:v>USER_NOT_ACTIVE</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
-        <x:v>Lệnh này chưa được bật. Mã lỗi: {error_id}</x:v>
+        <x:v>Tài khoản chưa được cấp quyền hoạt động. Mã lỗi: {error_id}</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
         <x:v>vi-VN</x:v>
@@ -3169,9 +3169,23 @@
         <x:v>ACTIVE</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="9" t="str">
+        <x:v>COMMAND_NOT_AVAILABLE</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>Lệnh này chưa được bật. Mã lỗi: {error_id}</x:v>
+      </x:c>
+      <x:c r="C10" s="9" t="str">
+        <x:v>vi-VN</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
-    <x:dataValidation type="list" sqref="D2:D9">
+    <x:dataValidation type="list" sqref="D2:D10">
       <x:formula1>"ACTIVE,INACTIVE"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
fix: harden V2 config gateway status flow
</commit_message>
<xml_diff>
--- a/outputs/issue-2/KKB_V2_CONFIG_BASELINE.xlsx
+++ b/outputs/issue-2/KKB_V2_CONFIG_BASELINE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SCHEMA" sheetId="1" r:id="Rff5ee20d738c4112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_VERSION" sheetId="2" r:id="R3ed994e67de340b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_GLOBAL" sheetId="3" r:id="R0c681aac3625444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_BRANCH" sheetId="4" r:id="Rdd6e309094254020"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_USER" sheetId="5" r:id="R49de009770c54ac8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_THONG_BAO" sheetId="6" r:id="R4e3ee4fb76f6474f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SNAPSHOT" sheetId="7" r:id="R7a5890ca5b0a4f91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERATION" sheetId="8" r:id="R6757e33456b64429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERROR_BIA" sheetId="9" r:id="R210f965374cb4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SCHEMA" sheetId="1" r:id="R5ad5da092d0743b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_VERSION" sheetId="2" r:id="R89caffdd2cc74561"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_GLOBAL" sheetId="3" r:id="Rf58e48890b004ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_BRANCH" sheetId="4" r:id="Rde972767eae244fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_USER" sheetId="5" r:id="R379385a43e854a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_THONG_BAO" sheetId="6" r:id="R49381705ae244232"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONFIG_SNAPSHOT" sheetId="7" r:id="R5f29c326c1d449f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OPERATION" sheetId="8" r:id="R715f8407f0c04624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERROR_BIA" sheetId="9" r:id="R0bee2ab248674ce7"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>